<commit_message>
Dar formato a menu.xlsx: encabezado con color, anchos de columna y precios en formato moneda
</commit_message>
<xml_diff>
--- a/menu.xlsx
+++ b/menu.xlsx
@@ -28,8 +28,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,13 +39,23 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFBF4"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00614E4C"/>
+        <bgColor rgb="00614E4C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -58,8 +70,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,34 +443,42 @@
   </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>precio_s</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio_m</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_l</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_xl</t>
         </is>
@@ -471,16 +495,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>3300</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>4200</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>4800</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="2" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -495,16 +519,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>3300</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>4200</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>4800</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="2" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -519,16 +543,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>3300</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>4200</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>4800</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="2" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -543,16 +567,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2" t="n">
         <v>3300</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>4200</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>4800</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="2" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -567,16 +591,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="2" t="n">
         <v>3300</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>4200</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>4800</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="2" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -591,16 +615,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="2" t="n">
         <v>3300</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>4200</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="2" t="n">
         <v>4800</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="2" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -615,16 +639,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="2" t="n">
         <v>3300</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
         <v>4200</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="2" t="n">
         <v>4800</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="2" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -639,16 +663,16 @@
           <t>si</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="2" t="n">
         <v>3300</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
         <v>4200</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="2" t="n">
         <v>4800</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="2" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -665,34 +689,42 @@
   </sheetPr>
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -714,9 +746,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>10800</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -734,9 +767,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>10800</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -754,9 +788,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>10800</v>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -774,9 +809,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>10800</v>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -794,9 +830,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>10800</v>
       </c>
+      <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -814,9 +851,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>10800</v>
       </c>
+      <c r="E7" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -831,34 +869,42 @@
   </sheetPr>
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -880,9 +926,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>7500</v>
       </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>torta-hawaiana.png</t>
@@ -905,9 +952,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>7500</v>
       </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>torta-agus-tina.png</t>
@@ -930,9 +978,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>7500</v>
       </c>
+      <c r="E4" s="2" t="n"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>torta-valen-tina.png</t>
@@ -955,9 +1004,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>7500</v>
       </c>
+      <c r="E5" s="2" t="n"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>torta-capricho.png</t>
@@ -980,9 +1030,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>7500</v>
       </c>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>torta-brownie-boom.png</t>
@@ -1005,9 +1056,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>7500</v>
       </c>
+      <c r="E7" s="2" t="n"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>torta-banofee.png</t>
@@ -1027,34 +1079,42 @@
   </sheetPr>
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -1076,9 +1136,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>14400</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1096,9 +1157,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>13800</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1116,9 +1178,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>10800</v>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1136,9 +1199,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>10700</v>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1153,34 +1217,42 @@
   </sheetPr>
   <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -1202,9 +1274,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>7800</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1222,9 +1295,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>9000</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1242,9 +1316,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>8300</v>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1262,9 +1337,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>8000</v>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1282,9 +1358,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>14500</v>
       </c>
+      <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1302,9 +1379,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>13800</v>
       </c>
+      <c r="E7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1322,9 +1400,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
         <v>12800</v>
       </c>
+      <c r="E8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1342,9 +1421,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
         <v>16000</v>
       </c>
+      <c r="E9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1362,9 +1442,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="2" t="n">
         <v>16600</v>
       </c>
+      <c r="E10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1382,9 +1463,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="2" t="n">
         <v>17400</v>
       </c>
+      <c r="E11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1402,9 +1484,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="2" t="n">
         <v>12800</v>
       </c>
+      <c r="E12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1422,9 +1505,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="2" t="n">
         <v>17400</v>
       </c>
+      <c r="E13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1442,9 +1526,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="2" t="n">
         <v>37200</v>
       </c>
+      <c r="E14" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1459,34 +1544,42 @@
   </sheetPr>
   <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -1508,9 +1601,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1523,9 +1617,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1538,9 +1633,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1553,9 +1649,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1568,9 +1665,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1583,9 +1681,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1598,9 +1697,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1618,9 +1718,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1633,9 +1734,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1648,9 +1750,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1663,9 +1766,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1678,9 +1782,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1693,9 +1798,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E14" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1710,34 +1816,42 @@
   </sheetPr>
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -1759,9 +1873,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>4600</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1779,9 +1894,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>4900</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1796,34 +1912,42 @@
   </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -1840,9 +1964,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>6600</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1855,9 +1980,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>6600</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1870,9 +1996,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>6600</v>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1885,9 +2012,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>6600</v>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1900,9 +2028,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>6600</v>
       </c>
+      <c r="E6" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1917,34 +2046,42 @@
   </sheetPr>
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -1961,9 +2098,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>6000</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1976,9 +2114,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>3300</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1991,9 +2130,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>3300</v>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2011,9 +2151,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>6400</v>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2028,34 +2169,42 @@
   </sheetPr>
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -2072,9 +2221,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>6600</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2087,9 +2237,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>6600</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2102,9 +2253,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>6600</v>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2117,9 +2269,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>6600</v>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2134,34 +2287,42 @@
   </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -2178,9 +2339,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>4100</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2198,9 +2360,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>4100</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2213,10 +2376,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>6000</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>7600</v>
       </c>
     </row>
@@ -2231,9 +2394,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>8700</v>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2251,10 +2415,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>8700</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>9600</v>
       </c>
     </row>
@@ -2271,34 +2435,42 @@
   </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -2315,9 +2487,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>7100</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2330,9 +2503,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>7100</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2345,9 +2519,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>7100</v>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2360,9 +2535,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>7100</v>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2375,9 +2551,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>7100</v>
       </c>
+      <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2390,9 +2567,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>7100</v>
       </c>
+      <c r="E7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2405,9 +2583,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
         <v>7100</v>
       </c>
+      <c r="E8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2420,9 +2599,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
         <v>7100</v>
       </c>
+      <c r="E9" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2437,34 +2617,42 @@
   </sheetPr>
   <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>descripcion</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>disponible</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
@@ -2486,9 +2674,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>6600</v>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2501,9 +2690,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>4200</v>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2521,9 +2711,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>2800</v>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2541,9 +2732,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>2800</v>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2556,9 +2748,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>2800</v>
       </c>
+      <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2571,9 +2764,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>7000</v>
       </c>
+      <c r="E7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2586,9 +2780,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
         <v>3500</v>
       </c>
+      <c r="E8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2606,9 +2801,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
         <v>3600</v>
       </c>
+      <c r="E9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2621,9 +2817,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="2" t="n">
         <v>850</v>
       </c>
+      <c r="E10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2636,9 +2833,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="2" t="n">
         <v>9200</v>
       </c>
+      <c r="E11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2656,10 +2854,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="2" t="n">
         <v>1400</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="2" t="n">
         <v>3300</v>
       </c>
     </row>
@@ -2674,9 +2872,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="2" t="n">
         <v>9200</v>
       </c>
+      <c r="E13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2689,9 +2888,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="2" t="n">
         <v>9200</v>
       </c>
+      <c r="E14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2709,9 +2909,10 @@
           <t>si</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="2" t="n">
         <v>2100</v>
       </c>
+      <c r="E15" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Hacer editable el precio del tazón extra de promos desde menu.xlsx
</commit_message>
<xml_diff>
--- a/menu.xlsx
+++ b/menu.xlsx
@@ -1215,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1530,6 +1530,27 @@
         <v>37200</v>
       </c>
       <c r="E14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Agrandá a tazón (extra)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>no es una promo de la grilla: alimenta el cartel "agrandá tus promos a tazón por $..."</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E15" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Separar la constante del tazón extra en columnas propias, fuera de la tabla de promos
</commit_message>
<xml_diff>
--- a/menu.xlsx
+++ b/menu.xlsx
@@ -1215,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1224,6 +1224,8 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1257,6 +1259,16 @@
           <t>imagen</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>nombre_constante</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>precio_constante</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1278,6 +1290,14 @@
         <v>7800</v>
       </c>
       <c r="E2" s="2" t="n"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Agrandá a tazón (extra)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>1500</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1530,27 +1550,6 @@
         <v>37200</v>
       </c>
       <c r="E14" s="2" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Agrandá a tazón (extra)</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>no es una promo de la grilla: alimenta el cartel "agrandá tus promos a tazón por $..."</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E15" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Agregar columna compartir explícita en Promos y bordes/alineación para mejor lectura en Sheets
</commit_message>
<xml_diff>
--- a/menu.xlsx
+++ b/menu.xlsx
@@ -58,7 +58,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -66,16 +66,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D2C7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D2C7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D2C7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D2C7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -485,194 +503,194 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Expresso</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>3300</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="4" t="n">
         <v>4200</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="4" t="n">
         <v>5500</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Doble Expresso</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>3300</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="4" t="n">
         <v>4200</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="4" t="n">
         <v>5500</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Café con leche</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>3300</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="4" t="n">
         <v>4200</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="4" t="n">
         <v>5500</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Cortado</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>3300</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="4" t="n">
         <v>4200</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="4" t="n">
         <v>5500</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Lágrima</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>3300</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="4" t="n">
         <v>4200</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="4" t="n">
         <v>5500</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Expresso Panna</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>3300</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="4" t="n">
         <v>4200</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="4" t="n">
         <v>5500</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Ice Coffee</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>3300</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="4" t="n">
         <v>4200</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="4" t="n">
         <v>5500</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Expresso Tonic</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="n">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>3300</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="4" t="n">
         <v>4200</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="4" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -687,15 +705,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -716,145 +735,186 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Serrano</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>rúcula, jamón crudo y nueces</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>10800</v>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Azul</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>queso untable, queso roquefort y tomate hidratado</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>10800</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Gourmet</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>peras, queso azul, rúcula, nueces y miel</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>10800</v>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Capresse</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>tomate, queso y albahaca</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>10800</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Tradicional</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>jamón, queso, lechuga y tomate</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>10800</v>
       </c>
-      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Fugazza</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>queso y cebolla caramelizada</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>10800</v>
       </c>
-      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -867,15 +927,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -896,171 +957,206 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Hawaiana</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>mousse de coco y corazón de ananá</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>7500</v>
       </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>torta-hawaiana.png</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Agus Tina</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>mousse de chocolate, centro de naranja, terciopelo de chocolate</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>7500</v>
       </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>torta-agus-tina.png</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Valen Tina</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>profiterol relleno de cheesecake de pistacho, centro de praline de pistacho</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>7500</v>
       </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>torta-valen-tina.png</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Capricho</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>cremoso de chocolate, centro de maracuyá y frambuesa, terciopelo de chocolate blanco</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>7500</v>
       </c>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>torta-capricho.png</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Brownie boom</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>húmedo de chocolate, pasta de maní y dulce de leche, bañado en chocolate y crocante de maní</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>7500</v>
       </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>torta-brownie-boom.png</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Banofee</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>base de chocolate, ganache de maní, bananas caramelizadas, salsa toffee y mousse de chocolate</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>7500</v>
       </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>torta-banofee.png</t>
         </is>
@@ -1077,15 +1173,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1106,103 +1203,132 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Americano</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Cafetería + jugo exprimido + pan de campo con palta y huevo</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>14400</v>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Tentación</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Café con leche + jugo exprimido + opción de pastelería</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>13800</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Criollo</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Cafetería + jugo exprimido + tostadas con queso, manteca o dulce</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>10800</v>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Alfajor</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Cafetería + jugo exprimido + alfajor</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>10700</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1215,17 +1341,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1246,310 +1373,393 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>nombre_constante</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>precio_constante</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Clásico</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Infusión cafetería + 2 medialunas o tostadas + jugo</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>7800</v>
       </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="H2" t="inlineStr">
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Agrandá a tazón (extra)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="J2" s="4" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Minis</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Chocolatada / Jugo mediano + cookies / sandwich</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>9000</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Criollo</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Infusión cafetería + tostada con manteca o queso y dulce + jugo</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>8300</v>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Alfajor</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Infusión cafetería + alfajor a elección + jugo</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>8000</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Tentación</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Café especial + porción de torta + jugo</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>14500</v>
       </c>
-      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Saludable</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Infusión cafetería + yogurt con granola + frutillas y arándanos + jugo</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>13800</v>
       </c>
-      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Americano</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Infusión cafetería + tostada con huevo y palta + jugo</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>12800</v>
       </c>
-      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Stella</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Cerveza + focaccia a elección</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
         <v>16000</v>
       </c>
-      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Carlitos</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Infusión cafetería + tostada con jamón y queso + jugo</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
         <v>16600</v>
       </c>
-      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Gran Americano</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Infusión cafetería + jamón, queso y huevo + mix de frutas + tostadas + jugo</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
         <v>17400</v>
       </c>
-      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Trío Macarons</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Té en hebras / Infusión cafetería + jugo + trío de macarons</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
         <v>12800</v>
       </c>
-      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Tina</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Tetera té en hebras + 2 porciones budín + 2 scones + madeleine + financieros + 2 jugos (para compartir)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="n">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Tetera té en hebras + 2 porciones budín + 2 scones + madeleine + financieros + 2 jugos</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
         <v>17400</v>
       </c>
-      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Degustación</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>jarra de limonada a elección + degustación de focaccia (para compartir)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>jarra de limonada a elección + degustación de focaccia</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>37200</v>
       </c>
-      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1562,15 +1772,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1591,237 +1802,331 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Capuccino</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Clásico / Frambuesa</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Café Moccha Vienés</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Caramel Macchiato</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Macchiato Avellanas</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Café Irlandés</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Latte Vainilla</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Affogato</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Iced Coffee</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Pistacho / Coco</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Café Tina</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Café Bombón</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Café caribeño</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Submarino</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="n">
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Bayleis</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1834,15 +2139,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1863,61 +2169,78 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Jaguar / Pampa / Paradise</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>mate + blend yerba a elección + termo 80°</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>4600</v>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Opción Tereré</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>mate + blend yerba a elección + termo 80°</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>4900</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1930,15 +2253,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1959,99 +2283,139 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Banana con dulce de leche</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>6600</v>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Arándanos</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>6600</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Frutos rojos</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>6600</v>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Frutillas con crema</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>6600</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Mousse de limón</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>6600</v>
       </c>
-      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2064,15 +2428,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2093,88 +2458,120 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Tetera para compartir</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>6000</v>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Tetera individual</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>3300</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Té / Yerbeado</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>3300</v>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Matcha latte</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>té verde en polvo con leche</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>6400</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2187,15 +2584,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2216,83 +2614,116 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Café bombón</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>6600</v>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Mocha Vainilla Latte</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>6600</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Caramel Avellanas</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>6600</v>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Frambuesa</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>6600</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2305,15 +2736,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2334,113 +2766,151 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Agua / Agua Saborizada</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>4100</v>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Gaseosas</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Línea Pepsi</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>4100</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Jugo natural de naranja</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>6000</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="F4" s="4" t="n">
         <v>7600</v>
       </c>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Pomelada</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>8700</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Limonada</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Clásica / Menta jengibre / Arándanos / Maracuyá / Cereza</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>8700</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="F6" s="4" t="n">
         <v>9600</v>
       </c>
+      <c r="G6" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2453,15 +2923,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2482,147 +2953,208 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Brownie con frutos rojos</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>7100</v>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Crumble</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>7100</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Cheesecake</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>7100</v>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Balcarce</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>7100</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Selva Negra</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>7100</v>
       </c>
-      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Lemon Pie</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>7100</v>
       </c>
-      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Limón Cocado</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>7100</v>
       </c>
-      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Tiramisú</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
         <v>7100</v>
       </c>
-      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2635,15 +3167,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2664,275 +3197,372 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>compartir</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>precio_2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>imagen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Alfajores Premium</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Pistacho / Red Velvet / Chocotorta</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>6600</v>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Alfajor Maicena / Miel</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>4200</v>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Financieros</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>4 unidades</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>2800</v>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Madeleine</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>3 unidades</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>2800</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Cookies</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>2800</v>
       </c>
-      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Macarons</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>7000</v>
       </c>
-      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Budín</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>3500</v>
       </c>
-      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Scones</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>3 unidades</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
         <v>3600</v>
       </c>
-      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Tortita</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
         <v>850</v>
       </c>
-      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Tostado jamón y queso</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
         <v>9200</v>
       </c>
-      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Medialuna</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>opc. jamón y queso</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
         <v>1400</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="F12" s="4" t="n">
         <v>3300</v>
       </c>
+      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Tostón con omelette</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="n">
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
         <v>9200</v>
       </c>
-      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Bruschetta Tina</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>9200</v>
       </c>
-      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Galletas Bretón</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>3 unidades</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="n">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
         <v>2100</v>
       </c>
-      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="4" t="n"/>
+      <c r="G15" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>